<commit_message>
Add contact templates, results dashboard and progress log
- New Excel sheet 'Mensajes de contacto': WhatsApp/email/visit templates for Anillo 1
- New Excel sheet 'Tablero y Resultados': live funnel (COUNTIF on Estado column),
  close rate, breakdown by priority and ring, weekly logbook
- PROGRESO-FERRETERIAS.md: running tracker to review results week by week

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012DrgrVepVdHgyXphRTNJmB
</commit_message>
<xml_diff>
--- a/data/Ferreterias-CABA-Uniproveedores.xlsx
+++ b/data/Ferreterias-CABA-Uniproveedores.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Cómo completar y escalar" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Plan Semanal Redes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Seguidores por Red" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Mensajes de contacto" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tablero y Resultados" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ferreterías CABA'!$A$3:$O$81</definedName>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +70,16 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -101,6 +111,11 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F7E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -128,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -177,6 +192,26 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5411,4 +5446,454 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Plantillas de contacto — Anillo 1 (Comuna 10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Personalizá lo que está entre [corchetes]. Regla: mensaje corto, valor claro, una sola pregunta y CTA. No mandar catálogo entero en el primer mensaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="11" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1) WhatsApp — primer mensaje (frío)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Hola, ¿cómo va? Te escribo de UNIPROVEEDORES 🛠️, distribuidora mayorista de herramientas y artículos de ferretería. Estamos trabajando con ferreterías de [barrio/zona] con precio mayorista, envío y garantía. ¿Con quién puedo hablar por las compras? Te acerco la lista y las ofertas de la semana, sin compromiso. ¡Gracias!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2) WhatsApp — seguimiento (48-72 hs después, si no respondió)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="92" customHeight="1">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Hola [nombre]! Te escribí hace unos días de Uniproveedores (mayorista de ferretería). ¿Pudiste ver? Si querés te paso la lista de precios actualizada de esta semana. Si hay algún producto puntual que más vendés, decime cuál y te coto al toque 👍</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3) WhatsApp — con oferta gancho (si sabés qué vende)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="92" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Hola [nombre]! Esta semana tenemos [producto] a $[precio] mayorista (con envío y garantía). Es de lo que más rota en ferretería. ¿Te preparo una cotización con cantidades para [nombre de la ferretería]?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4) Email — presentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Asunto:  Uniproveedores — precios mayoristas para tu ferretería (envío y garantía)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="92" customHeight="1">
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Hola, ¿cómo estás?
+Soy [tu nombre], de UNIPROVEEDORES, distribuidora mayorista de herramientas y artículos de ferretería. Trabajamos con ferreterías de Capital con precio mayorista, envío y garantía por Mercado Libre.
+Me gustaría acercarte nuestra lista de precios y las ofertas de la semana, sin compromiso. ¿A quién le puedo enviar la información de compras?
+Quedo a disposición.
+[tu nombre] — Uniproveedores
+WhatsApp: 011-3551-0715  ·  ventas@distribuidorauniverso.com
+uniproveedores.com.ar  ·  Mercado Libre: /tienda/uniproveedores</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5) Guion visita / llamada (para conseguir el nombre del encargado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="92" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Buenas, ¿el encargado de compras se encuentra? Soy de Uniproveedores, distribuidora mayorista de ferretería. Le quería dejar la lista de precios y ver qué productos le interesan para cotizarle con envío. ¿Con quién tengo el gusto? (→ anotar el nombre en la columna 'Encargado').</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Tips de cierre:</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Guardá cada número que contactás como contacto → así ven tu foto/estado de empresa y da confianza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Después del primer 'sí', mandá SIEMPRE una cotización concreta con cantidades, no una lista genérica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Invitá a cada contacto a tu Canal de WhatsApp (ofertas) aunque todavía no te compre.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>UNIPROVEEDORES · Tablero de resultados (se actualiza al cargar la columna 'Estado')</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Embudo de prospección</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>Sin contactar</t>
+        </is>
+      </c>
+      <c r="C4" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Sin contactar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Contactado</t>
+        </is>
+      </c>
+      <c r="C5" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Contactado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Interesado</t>
+        </is>
+      </c>
+      <c r="C6" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Interesado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Cotización enviada</t>
+        </is>
+      </c>
+      <c r="C7" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Cotización enviada")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="C8" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Descartado</t>
+        </is>
+      </c>
+      <c r="C9" s="21">
+        <f>COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Descartado")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL en la lista</t>
+        </is>
+      </c>
+      <c r="C10" s="23">
+        <f>COUNTA('Ferreterías CABA'!$M$4:$M$81)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Tasa de cierre (Cliente / Contactadas+)</t>
+        </is>
+      </c>
+      <c r="C12" s="25">
+        <f>IFERROR(COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Cliente")/(COUNTA('Ferreterías CABA'!$M$4:$M$81)-COUNTIF('Ferreterías CABA'!$M$4:$M$81,"Sin contactar")-COUNTIF('Ferreterías CABA'!$M$4:$M$81,"")),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Por prioridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C15" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$N$4:$N$81,"Alta")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="C16" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$N$4:$N$81,"Media")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="C17" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$N$4:$N$81,"Baja")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Por anillo (cercanía al depósito)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Anillo 1</t>
+        </is>
+      </c>
+      <c r="C20" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$B$4:$B$81,"Anillo 1")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Anillo 2</t>
+        </is>
+      </c>
+      <c r="C21" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$B$4:$B$81,"Anillo 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Anillo 3</t>
+        </is>
+      </c>
+      <c r="C22" s="26">
+        <f>COUNTIF('Ferreterías CABA'!$B$4:$B$81,"Anillo 3")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Bitácora semanal (anotá a mano)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Contactadas</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Notas / aprendizajes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Semana 1</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="27" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>Semana 2</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>Semana 3</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="27" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>Semana 4</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="27" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>Semana 5</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="n"/>
+      <c r="D31" s="27" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>Semana 6</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="27" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Semana 7</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="n"/>
+      <c r="D33" s="27" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>Semana 8</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="n"/>
+      <c r="D34" s="27" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>